<commit_message>
Add June 6 screener output with WPS scoring
Fresh run with Winner-Pattern Score integrated. Includes balance-sheet
gate fix (catches thin-cash-cushion diluters) and tailwind calibration
(tag-driven, no trailing CAGR drag on turnarounds). 30 stocks across
3 tiers.

https://claude.ai/code/session_01JddThw18de4GoJHnFCFNA6
</commit_message>
<xml_diff>
--- a/output/screener_output_20260606.xlsx
+++ b/output/screener_output_20260606.xlsx
@@ -208,17 +208,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E76F51"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00B5D8B0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4E4B0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E76F51"/>
       </patternFill>
     </fill>
     <fill>
@@ -539,10 +539,13 @@
     <xf numFmtId="165" fontId="10" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="7" fillId="11" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="11" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="8" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -560,13 +563,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -618,7 +618,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="18" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -630,16 +630,16 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="13" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="12" fillId="13" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="12" fillId="13" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="13" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -682,19 +682,19 @@
     <xf numFmtId="164" fontId="15" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="13" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="13" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="13" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="12" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="12" fillId="13" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3573,25 +3573,25 @@
           <t>Nano Cap</t>
         </is>
       </c>
-      <c r="E17" s="41" t="n">
+      <c r="E17" s="42" t="n">
         <v>86.8</v>
       </c>
-      <c r="F17" s="41" t="n">
+      <c r="F17" s="42" t="n">
         <v>84.90000000000001</v>
       </c>
-      <c r="G17" s="41" t="n">
+      <c r="G17" s="42" t="n">
         <v>87.90000000000001</v>
       </c>
-      <c r="H17" s="41" t="n">
+      <c r="H17" s="42" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="I17" s="41" t="n">
+      <c r="I17" s="42" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="J17" s="41" t="n">
+      <c r="J17" s="42" t="n">
         <v>84.90000000000001</v>
       </c>
-      <c r="K17" s="41" t="n">
+      <c r="K17" s="42" t="n">
         <v>5.5</v>
       </c>
       <c r="L17" s="27" t="inlineStr">
@@ -3659,25 +3659,25 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E19" s="41" t="n">
+      <c r="E19" s="42" t="n">
         <v>82.59999999999999</v>
       </c>
-      <c r="F19" s="41" t="n">
+      <c r="F19" s="42" t="n">
         <v>79.5</v>
       </c>
-      <c r="G19" s="41" t="n">
+      <c r="G19" s="42" t="n">
         <v>85.8</v>
       </c>
-      <c r="H19" s="41" t="n">
+      <c r="H19" s="42" t="n">
         <v>85.8</v>
       </c>
-      <c r="I19" s="41" t="n">
+      <c r="I19" s="42" t="n">
         <v>85.8</v>
       </c>
-      <c r="J19" s="41" t="n">
+      <c r="J19" s="42" t="n">
         <v>79.5</v>
       </c>
-      <c r="K19" s="41" t="n">
+      <c r="K19" s="42" t="n">
         <v>6.299999999999997</v>
       </c>
       <c r="L19" s="27" t="inlineStr">
@@ -3745,25 +3745,25 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E21" s="41" t="n">
+      <c r="E21" s="42" t="n">
         <v>81.7</v>
       </c>
-      <c r="F21" s="41" t="n">
+      <c r="F21" s="42" t="n">
         <v>81.90000000000001</v>
       </c>
-      <c r="G21" s="41" t="n">
+      <c r="G21" s="42" t="n">
         <v>81</v>
       </c>
-      <c r="H21" s="41" t="n">
+      <c r="H21" s="42" t="n">
         <v>82.40000000000001</v>
       </c>
-      <c r="I21" s="41" t="n">
+      <c r="I21" s="42" t="n">
         <v>82.40000000000001</v>
       </c>
-      <c r="J21" s="41" t="n">
+      <c r="J21" s="42" t="n">
         <v>81</v>
       </c>
-      <c r="K21" s="41" t="n">
+      <c r="K21" s="42" t="n">
         <v>1.400000000000006</v>
       </c>
       <c r="L21" s="27" t="inlineStr">
@@ -3831,28 +3831,28 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E23" s="41" t="n">
+      <c r="E23" s="42" t="n">
         <v>81.2</v>
       </c>
-      <c r="F23" s="41" t="n">
+      <c r="F23" s="42" t="n">
         <v>84.3</v>
       </c>
-      <c r="G23" s="41" t="n">
+      <c r="G23" s="42" t="n">
         <v>79.5</v>
       </c>
-      <c r="H23" s="41" t="n">
+      <c r="H23" s="42" t="n">
         <v>73.5</v>
       </c>
-      <c r="I23" s="41" t="n">
+      <c r="I23" s="42" t="n">
         <v>84.3</v>
       </c>
-      <c r="J23" s="41" t="n">
+      <c r="J23" s="42" t="n">
         <v>73.5</v>
       </c>
-      <c r="K23" s="41" t="n">
+      <c r="K23" s="42" t="n">
         <v>10.8</v>
       </c>
-      <c r="L23" s="45" t="inlineStr">
+      <c r="L23" s="46" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -3917,25 +3917,25 @@
           <t>Nano Cap</t>
         </is>
       </c>
-      <c r="E25" s="41" t="n">
+      <c r="E25" s="42" t="n">
         <v>80.7</v>
       </c>
-      <c r="F25" s="41" t="n">
+      <c r="F25" s="42" t="n">
         <v>79.5</v>
       </c>
-      <c r="G25" s="41" t="n">
+      <c r="G25" s="42" t="n">
         <v>82.2</v>
       </c>
-      <c r="H25" s="41" t="n">
+      <c r="H25" s="42" t="n">
         <v>82.2</v>
       </c>
-      <c r="I25" s="41" t="n">
+      <c r="I25" s="42" t="n">
         <v>82.2</v>
       </c>
-      <c r="J25" s="41" t="n">
+      <c r="J25" s="42" t="n">
         <v>79.5</v>
       </c>
-      <c r="K25" s="41" t="n">
+      <c r="K25" s="42" t="n">
         <v>2.700000000000003</v>
       </c>
       <c r="L25" s="27" t="inlineStr">
@@ -4003,25 +4003,25 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E27" s="41" t="n">
+      <c r="E27" s="42" t="n">
         <v>79.8</v>
       </c>
-      <c r="F27" s="41" t="n">
+      <c r="F27" s="42" t="n">
         <v>80</v>
       </c>
-      <c r="G27" s="41" t="n">
+      <c r="G27" s="42" t="n">
         <v>80.5</v>
       </c>
-      <c r="H27" s="41" t="n">
+      <c r="H27" s="42" t="n">
         <v>76.8</v>
       </c>
-      <c r="I27" s="41" t="n">
+      <c r="I27" s="42" t="n">
         <v>80.5</v>
       </c>
-      <c r="J27" s="41" t="n">
+      <c r="J27" s="42" t="n">
         <v>76.8</v>
       </c>
-      <c r="K27" s="41" t="n">
+      <c r="K27" s="42" t="n">
         <v>3.700000000000003</v>
       </c>
       <c r="L27" s="27" t="inlineStr">
@@ -4089,25 +4089,25 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E29" s="41" t="n">
+      <c r="E29" s="42" t="n">
         <v>78.90000000000001</v>
       </c>
-      <c r="F29" s="41" t="n">
+      <c r="F29" s="42" t="n">
         <v>74.5</v>
       </c>
-      <c r="G29" s="41" t="n">
+      <c r="G29" s="42" t="n">
         <v>83.8</v>
       </c>
-      <c r="H29" s="41" t="n">
+      <c r="H29" s="42" t="n">
         <v>81.90000000000001</v>
       </c>
-      <c r="I29" s="41" t="n">
+      <c r="I29" s="42" t="n">
         <v>83.8</v>
       </c>
-      <c r="J29" s="41" t="n">
+      <c r="J29" s="42" t="n">
         <v>74.5</v>
       </c>
-      <c r="K29" s="41" t="n">
+      <c r="K29" s="42" t="n">
         <v>9.299999999999997</v>
       </c>
       <c r="L29" s="27" t="inlineStr">
@@ -4175,25 +4175,25 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E31" s="41" t="n">
+      <c r="E31" s="42" t="n">
         <v>77.59999999999999</v>
       </c>
-      <c r="F31" s="41" t="n">
+      <c r="F31" s="42" t="n">
         <v>79.8</v>
       </c>
-      <c r="G31" s="41" t="n">
+      <c r="G31" s="42" t="n">
         <v>76.5</v>
       </c>
-      <c r="H31" s="41" t="n">
+      <c r="H31" s="42" t="n">
         <v>71.40000000000001</v>
       </c>
-      <c r="I31" s="41" t="n">
+      <c r="I31" s="42" t="n">
         <v>79.8</v>
       </c>
-      <c r="J31" s="41" t="n">
+      <c r="J31" s="42" t="n">
         <v>71.40000000000001</v>
       </c>
-      <c r="K31" s="41" t="n">
+      <c r="K31" s="42" t="n">
         <v>8.399999999999991</v>
       </c>
       <c r="L31" s="27" t="inlineStr">
@@ -4261,25 +4261,25 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E33" s="41" t="n">
+      <c r="E33" s="42" t="n">
         <v>76.7</v>
       </c>
-      <c r="F33" s="41" t="n">
+      <c r="F33" s="42" t="n">
         <v>72.7</v>
       </c>
-      <c r="G33" s="41" t="n">
+      <c r="G33" s="42" t="n">
         <v>80.7</v>
       </c>
-      <c r="H33" s="41" t="n">
+      <c r="H33" s="42" t="n">
         <v>80.7</v>
       </c>
-      <c r="I33" s="41" t="n">
+      <c r="I33" s="42" t="n">
         <v>80.7</v>
       </c>
-      <c r="J33" s="41" t="n">
+      <c r="J33" s="42" t="n">
         <v>72.7</v>
       </c>
-      <c r="K33" s="41" t="n">
+      <c r="K33" s="42" t="n">
         <v>8</v>
       </c>
       <c r="L33" s="27" t="inlineStr">
@@ -4347,25 +4347,25 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E35" s="41" t="n">
+      <c r="E35" s="42" t="n">
         <v>75.8</v>
       </c>
-      <c r="F35" s="41" t="n">
+      <c r="F35" s="42" t="n">
         <v>71.40000000000001</v>
       </c>
-      <c r="G35" s="41" t="n">
+      <c r="G35" s="42" t="n">
         <v>79.90000000000001</v>
       </c>
-      <c r="H35" s="41" t="n">
+      <c r="H35" s="42" t="n">
         <v>81.09999999999999</v>
       </c>
-      <c r="I35" s="41" t="n">
+      <c r="I35" s="42" t="n">
         <v>81.09999999999999</v>
       </c>
-      <c r="J35" s="41" t="n">
+      <c r="J35" s="42" t="n">
         <v>71.40000000000001</v>
       </c>
-      <c r="K35" s="41" t="n">
+      <c r="K35" s="42" t="n">
         <v>9.699999999999989</v>
       </c>
       <c r="L35" s="27" t="inlineStr">
@@ -4433,25 +4433,25 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E37" s="41" t="n">
+      <c r="E37" s="42" t="n">
         <v>75</v>
       </c>
-      <c r="F37" s="41" t="n">
+      <c r="F37" s="42" t="n">
         <v>71.7</v>
       </c>
-      <c r="G37" s="41" t="n">
+      <c r="G37" s="42" t="n">
         <v>78.40000000000001</v>
       </c>
-      <c r="H37" s="41" t="n">
+      <c r="H37" s="42" t="n">
         <v>78.40000000000001</v>
       </c>
-      <c r="I37" s="41" t="n">
+      <c r="I37" s="42" t="n">
         <v>78.40000000000001</v>
       </c>
-      <c r="J37" s="41" t="n">
+      <c r="J37" s="42" t="n">
         <v>71.7</v>
       </c>
-      <c r="K37" s="41" t="n">
+      <c r="K37" s="42" t="n">
         <v>6.700000000000003</v>
       </c>
       <c r="L37" s="27" t="inlineStr">
@@ -4519,25 +4519,25 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E39" s="41" t="n">
+      <c r="E39" s="42" t="n">
         <v>74.3</v>
       </c>
-      <c r="F39" s="41" t="n">
+      <c r="F39" s="42" t="n">
         <v>74.8</v>
       </c>
-      <c r="G39" s="41" t="n">
+      <c r="G39" s="42" t="n">
         <v>75.09999999999999</v>
       </c>
-      <c r="H39" s="41" t="n">
+      <c r="H39" s="42" t="n">
         <v>68.90000000000001</v>
       </c>
-      <c r="I39" s="41" t="n">
+      <c r="I39" s="42" t="n">
         <v>75.09999999999999</v>
       </c>
-      <c r="J39" s="41" t="n">
+      <c r="J39" s="42" t="n">
         <v>68.90000000000001</v>
       </c>
-      <c r="K39" s="41" t="n">
+      <c r="K39" s="42" t="n">
         <v>6.199999999999989</v>
       </c>
       <c r="L39" s="27" t="inlineStr">
@@ -4605,28 +4605,28 @@
           <t>Nano Cap</t>
         </is>
       </c>
-      <c r="E41" s="41" t="n">
+      <c r="E41" s="42" t="n">
         <v>73.90000000000001</v>
       </c>
-      <c r="F41" s="41" t="n">
+      <c r="F41" s="42" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="G41" s="41" t="n">
+      <c r="G41" s="42" t="n">
         <v>81.5</v>
       </c>
-      <c r="H41" s="41" t="n">
+      <c r="H41" s="42" t="n">
         <v>81.5</v>
       </c>
-      <c r="I41" s="41" t="n">
+      <c r="I41" s="42" t="n">
         <v>81.5</v>
       </c>
-      <c r="J41" s="41" t="n">
+      <c r="J41" s="42" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="K41" s="41" t="n">
+      <c r="K41" s="42" t="n">
         <v>15.09999999999999</v>
       </c>
-      <c r="L41" s="45" t="inlineStr">
+      <c r="L41" s="46" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -4691,25 +4691,25 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E43" s="41" t="n">
+      <c r="E43" s="42" t="n">
         <v>72</v>
       </c>
-      <c r="F43" s="41" t="n">
+      <c r="F43" s="42" t="n">
         <v>68</v>
       </c>
-      <c r="G43" s="41" t="n">
+      <c r="G43" s="42" t="n">
         <v>76.8</v>
       </c>
-      <c r="H43" s="41" t="n">
+      <c r="H43" s="42" t="n">
         <v>73.40000000000001</v>
       </c>
-      <c r="I43" s="41" t="n">
+      <c r="I43" s="42" t="n">
         <v>76.8</v>
       </c>
-      <c r="J43" s="41" t="n">
+      <c r="J43" s="42" t="n">
         <v>68</v>
       </c>
-      <c r="K43" s="41" t="n">
+      <c r="K43" s="42" t="n">
         <v>8.799999999999997</v>
       </c>
       <c r="L43" s="27" t="inlineStr">
@@ -4777,28 +4777,28 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E45" s="41" t="n">
+      <c r="E45" s="42" t="n">
         <v>71.09999999999999</v>
       </c>
-      <c r="F45" s="41" t="n">
+      <c r="F45" s="42" t="n">
         <v>65.7</v>
       </c>
-      <c r="G45" s="41" t="n">
+      <c r="G45" s="42" t="n">
         <v>76.90000000000001</v>
       </c>
-      <c r="H45" s="41" t="n">
+      <c r="H45" s="42" t="n">
         <v>75</v>
       </c>
-      <c r="I45" s="41" t="n">
+      <c r="I45" s="42" t="n">
         <v>76.90000000000001</v>
       </c>
-      <c r="J45" s="41" t="n">
+      <c r="J45" s="42" t="n">
         <v>65.7</v>
       </c>
-      <c r="K45" s="41" t="n">
+      <c r="K45" s="42" t="n">
         <v>11.2</v>
       </c>
-      <c r="L45" s="45" t="inlineStr">
+      <c r="L45" s="46" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -5065,7 +5065,7 @@
           <t>KULR  —  KULR Technology Group, Inc.</t>
         </is>
       </c>
-      <c r="C5" s="37" t="inlineStr">
+      <c r="C5" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -5256,7 +5256,7 @@
           <t>KVHI  —  KVH Industries, Inc.</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr">
+      <c r="C12" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -5447,7 +5447,7 @@
           <t>INTT  —  inTEST Corporation</t>
         </is>
       </c>
-      <c r="C19" s="37" t="inlineStr">
+      <c r="C19" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -5638,7 +5638,7 @@
           <t>CODA  —  Coda Octopus Group, Inc.</t>
         </is>
       </c>
-      <c r="C26" s="37" t="inlineStr">
+      <c r="C26" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -5829,7 +5829,7 @@
           <t>WSTL  —  Westell Technologies, Inc.</t>
         </is>
       </c>
-      <c r="C33" s="37" t="inlineStr">
+      <c r="C33" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -6020,7 +6020,7 @@
           <t>SCTQ  —  Spectra Systems Corporation</t>
         </is>
       </c>
-      <c r="C40" s="37" t="inlineStr">
+      <c r="C40" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -6194,7 +6194,7 @@
           <t>ESP  —  Espey Mfg. &amp; Electronics Corp.</t>
         </is>
       </c>
-      <c r="C47" s="37" t="inlineStr">
+      <c r="C47" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -6385,7 +6385,7 @@
           <t>BZAI  —  Blaize Holdings, Inc.</t>
         </is>
       </c>
-      <c r="C54" s="37" t="inlineStr">
+      <c r="C54" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -6576,7 +6576,7 @@
           <t>TAYD  —  Taylor Devices, Inc.</t>
         </is>
       </c>
-      <c r="C61" s="37" t="inlineStr">
+      <c r="C61" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -6767,7 +6767,7 @@
           <t>BYRN  —  Byrna Technologies Inc.</t>
         </is>
       </c>
-      <c r="C68" s="37" t="inlineStr">
+      <c r="C68" s="38" t="inlineStr">
         <is>
           <t>Nano Cap</t>
         </is>
@@ -6975,7 +6975,7 @@
           <t>DSP  —  Viant Technology Inc.</t>
         </is>
       </c>
-      <c r="C76" s="37" t="inlineStr">
+      <c r="C76" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -7166,7 +7166,7 @@
           <t>EVLV  —  Evolv Technologies Holdings, Inc.</t>
         </is>
       </c>
-      <c r="C83" s="37" t="inlineStr">
+      <c r="C83" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -7357,7 +7357,7 @@
           <t>PKE  —  Park Aerospace Corp.</t>
         </is>
       </c>
-      <c r="C90" s="37" t="inlineStr">
+      <c r="C90" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -7548,7 +7548,7 @@
           <t>CMCO  —  Columbus McKinnon Corporation</t>
         </is>
       </c>
-      <c r="C97" s="37" t="inlineStr">
+      <c r="C97" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -7739,7 +7739,7 @@
           <t>CDRE  —  Cadre Holdings, Inc.</t>
         </is>
       </c>
-      <c r="C104" s="37" t="inlineStr">
+      <c r="C104" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -7930,7 +7930,7 @@
           <t>ADTN  —  ADTRAN Holdings, Inc.</t>
         </is>
       </c>
-      <c r="C111" s="37" t="inlineStr">
+      <c r="C111" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -8121,7 +8121,7 @@
           <t>WYFI  —  WhiteFiber, Inc. Ordinary Shares</t>
         </is>
       </c>
-      <c r="C118" s="37" t="inlineStr">
+      <c r="C118" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -8312,7 +8312,7 @@
           <t>SWBI  —  Smith &amp; Wesson Brands, Inc.</t>
         </is>
       </c>
-      <c r="C125" s="37" t="inlineStr">
+      <c r="C125" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -8503,7 +8503,7 @@
           <t>ROCK  —  Gibraltar Industries, Inc.</t>
         </is>
       </c>
-      <c r="C132" s="37" t="inlineStr">
+      <c r="C132" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -8694,7 +8694,7 @@
           <t>BUKS  —  Butler National Corporation</t>
         </is>
       </c>
-      <c r="C139" s="37" t="inlineStr">
+      <c r="C139" s="38" t="inlineStr">
         <is>
           <t>Small Cap</t>
         </is>
@@ -8902,7 +8902,7 @@
           <t>KRMN  —  Karman Holdings Inc.</t>
         </is>
       </c>
-      <c r="C147" s="37" t="inlineStr">
+      <c r="C147" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -9093,7 +9093,7 @@
           <t>ESI  —  Element Solutions Inc</t>
         </is>
       </c>
-      <c r="C154" s="37" t="inlineStr">
+      <c r="C154" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -9284,7 +9284,7 @@
           <t>RUN  —  Sunrun Inc.</t>
         </is>
       </c>
-      <c r="C161" s="37" t="inlineStr">
+      <c r="C161" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -9475,7 +9475,7 @@
           <t>LYFT  —  Lyft, Inc.</t>
         </is>
       </c>
-      <c r="C168" s="37" t="inlineStr">
+      <c r="C168" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -9666,7 +9666,7 @@
           <t>FELE  —  Franklin Electric Co., Inc.</t>
         </is>
       </c>
-      <c r="C175" s="37" t="inlineStr">
+      <c r="C175" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -9857,7 +9857,7 @@
           <t>ALGM  —  Allegro MicroSystems, Inc.</t>
         </is>
       </c>
-      <c r="C182" s="37" t="inlineStr">
+      <c r="C182" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -10048,7 +10048,7 @@
           <t>IPGP  —  IPG Photonics Corporation</t>
         </is>
       </c>
-      <c r="C189" s="37" t="inlineStr">
+      <c r="C189" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -10239,7 +10239,7 @@
           <t>ESAB  —  ESAB Corporation</t>
         </is>
       </c>
-      <c r="C196" s="37" t="inlineStr">
+      <c r="C196" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -10430,7 +10430,7 @@
           <t>PINS  —  Pinterest, Inc.</t>
         </is>
       </c>
-      <c r="C203" s="37" t="inlineStr">
+      <c r="C203" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -10621,7 +10621,7 @@
           <t>RVTY  —  Revvity, Inc.</t>
         </is>
       </c>
-      <c r="C210" s="37" t="inlineStr">
+      <c r="C210" s="38" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
@@ -12426,13 +12426,13 @@
           <t>Gross Margin %</t>
         </is>
       </c>
-      <c r="B63" s="41" t="n">
+      <c r="B63" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="C63" s="41" t="n">
+      <c r="C63" s="42" t="n">
         <v>36.5</v>
       </c>
-      <c r="D63" s="41" t="n">
+      <c r="D63" s="42" t="n">
         <v>50</v>
       </c>
       <c r="E63" s="25" t="inlineStr">
@@ -12478,13 +12478,13 @@
           <t>Dilution 3yr %</t>
         </is>
       </c>
-      <c r="B65" s="41" t="n">
+      <c r="B65" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="C65" s="41" t="n">
+      <c r="C65" s="42" t="n">
         <v>7</v>
       </c>
-      <c r="D65" s="41" t="n">
+      <c r="D65" s="42" t="n">
         <v>25</v>
       </c>
       <c r="E65" s="25" t="inlineStr">
@@ -13260,15 +13260,15 @@
       <c r="M5" s="36" t="n">
         <v>91.3</v>
       </c>
-      <c r="N5" s="28" t="n">
-        <v>67.59999999999999</v>
-      </c>
-      <c r="O5" s="37" t="inlineStr">
+      <c r="N5" s="37" t="n">
+        <v>50</v>
+      </c>
+      <c r="O5" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P5" s="38" t="n">
+      <c r="P5" s="39" t="n">
         <v>15.6</v>
       </c>
       <c r="Q5" s="23" t="inlineStr">
@@ -13309,42 +13309,42 @@
       <c r="D6" s="26" t="n">
         <v>146.6</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="E6" s="40" t="n">
         <v>7.52</v>
       </c>
-      <c r="F6" s="40" t="n">
+      <c r="F6" s="41" t="n">
         <v>0.272</v>
       </c>
-      <c r="G6" s="40" t="n">
+      <c r="G6" s="41" t="n">
         <v>0.386</v>
       </c>
-      <c r="H6" s="40" t="n">
+      <c r="H6" s="41" t="n">
         <v>0.289</v>
       </c>
-      <c r="I6" s="40" t="n">
+      <c r="I6" s="41" t="n">
         <v>0.009000000000000001</v>
       </c>
-      <c r="J6" s="40" t="n">
+      <c r="J6" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="K6" s="41" t="n">
+      <c r="K6" s="42" t="n">
         <v>80.8</v>
       </c>
-      <c r="L6" s="41" t="n">
+      <c r="L6" s="42" t="n">
         <v>95.90000000000001</v>
       </c>
-      <c r="M6" s="42" t="n">
+      <c r="M6" s="43" t="n">
         <v>86.8</v>
       </c>
       <c r="N6" s="28" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="O6" s="43" t="inlineStr">
+        <v>66.5</v>
+      </c>
+      <c r="O6" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P6" s="38" t="n">
+      <c r="P6" s="39" t="n">
         <v>22.3</v>
       </c>
       <c r="Q6" s="27" t="inlineStr">
@@ -13352,19 +13352,19 @@
           <t>High</t>
         </is>
       </c>
-      <c r="R6" s="40" t="n">
+      <c r="R6" s="41" t="n">
         <v>-0.2025451</v>
       </c>
-      <c r="S6" s="40" t="n">
+      <c r="S6" s="41" t="n">
         <v>0.2533333</v>
       </c>
-      <c r="T6" s="40" t="n">
+      <c r="T6" s="41" t="n">
         <v>0.2368421</v>
       </c>
-      <c r="U6" s="40" t="n">
+      <c r="U6" s="41" t="n">
         <v>0.0789096</v>
       </c>
-      <c r="V6" s="40" t="n">
+      <c r="V6" s="41" t="n">
         <v>0.463035</v>
       </c>
     </row>
@@ -13413,14 +13413,14 @@
         <v>81.59999999999999</v>
       </c>
       <c r="N7" s="35" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="O7" s="37" t="inlineStr">
+        <v>40.8</v>
+      </c>
+      <c r="O7" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P7" s="44" t="n">
+      <c r="P7" s="45" t="n">
         <v>55.9</v>
       </c>
       <c r="Q7" s="23" t="inlineStr">
@@ -13461,42 +13461,42 @@
       <c r="D8" s="26" t="n">
         <v>133.1</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="E8" s="40" t="n">
         <v>11.8</v>
       </c>
-      <c r="F8" s="40" t="n">
+      <c r="F8" s="41" t="n">
         <v>0.288</v>
       </c>
-      <c r="G8" s="40" t="n">
+      <c r="G8" s="41" t="n">
         <v>0.309</v>
       </c>
-      <c r="H8" s="40" t="n">
+      <c r="H8" s="41" t="n">
         <v>0.6509999999999999</v>
       </c>
-      <c r="I8" s="40" t="n">
+      <c r="I8" s="41" t="n">
         <v>0.024</v>
       </c>
-      <c r="J8" s="40" t="n">
+      <c r="J8" s="41" t="n">
         <v>0.491</v>
       </c>
-      <c r="K8" s="41" t="n">
+      <c r="K8" s="42" t="n">
         <v>87.3</v>
       </c>
-      <c r="L8" s="41" t="n">
+      <c r="L8" s="42" t="n">
         <v>72.3</v>
       </c>
-      <c r="M8" s="42" t="n">
+      <c r="M8" s="43" t="n">
         <v>80.8</v>
       </c>
       <c r="N8" s="28" t="n">
-        <v>56.6</v>
-      </c>
-      <c r="O8" s="43" t="inlineStr">
+        <v>58</v>
+      </c>
+      <c r="O8" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P8" s="44" t="n">
+      <c r="P8" s="45" t="n">
         <v>41.2</v>
       </c>
       <c r="Q8" s="23" t="inlineStr">
@@ -13504,19 +13504,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R8" s="40" t="n">
+      <c r="R8" s="41" t="n">
         <v>0.0111397</v>
       </c>
-      <c r="S8" s="40" t="n">
+      <c r="S8" s="41" t="n">
         <v>-0.1559371</v>
       </c>
-      <c r="T8" s="40" t="n">
+      <c r="T8" s="41" t="n">
         <v>0.3736903</v>
       </c>
-      <c r="U8" s="40" t="n">
+      <c r="U8" s="41" t="n">
         <v>0.2688172</v>
       </c>
-      <c r="V8" s="40" t="n">
+      <c r="V8" s="41" t="n">
         <v>0.8910256</v>
       </c>
     </row>
@@ -13565,14 +13565,14 @@
         <v>80.7</v>
       </c>
       <c r="N9" s="28" t="n">
-        <v>54.5</v>
-      </c>
-      <c r="O9" s="37" t="inlineStr">
+        <v>57.3</v>
+      </c>
+      <c r="O9" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P9" s="44" t="n">
+      <c r="P9" s="45" t="n">
         <v>69.3</v>
       </c>
       <c r="Q9" s="23" t="inlineStr">
@@ -13613,42 +13613,42 @@
       <c r="D10" s="26" t="n">
         <v>101.7</v>
       </c>
-      <c r="E10" s="39" t="n">
+      <c r="E10" s="40" t="n">
         <v>2.13</v>
       </c>
-      <c r="F10" s="40" t="n">
+      <c r="F10" s="41" t="n">
         <v>5.018</v>
       </c>
-      <c r="G10" s="40" t="n">
+      <c r="G10" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="40" t="n">
+      <c r="H10" s="41" t="n">
         <v>0.57</v>
       </c>
-      <c r="I10" s="40" t="n">
+      <c r="I10" s="41" t="n">
         <v>0.052</v>
       </c>
-      <c r="J10" s="40" t="n">
+      <c r="J10" s="41" t="n">
         <v>0.179</v>
       </c>
-      <c r="K10" s="41" t="n">
+      <c r="K10" s="42" t="n">
         <v>84.8</v>
       </c>
-      <c r="L10" s="41" t="n">
+      <c r="L10" s="42" t="n">
         <v>73.3</v>
       </c>
-      <c r="M10" s="42" t="n">
+      <c r="M10" s="43" t="n">
         <v>80.2</v>
       </c>
       <c r="N10" s="28" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="O10" s="43" t="inlineStr">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="O10" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P10" s="38" t="n">
+      <c r="P10" s="39" t="n">
         <v>20.5</v>
       </c>
       <c r="Q10" s="23" t="inlineStr">
@@ -13656,19 +13656,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R10" s="40" t="n">
+      <c r="R10" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="S10" s="40" t="n">
+      <c r="S10" s="41" t="n">
         <v>0.0492611</v>
       </c>
-      <c r="T10" s="40" t="n">
+      <c r="T10" s="41" t="n">
         <v>0.0492611</v>
       </c>
-      <c r="U10" s="40" t="n">
+      <c r="U10" s="41" t="n">
         <v>0.0492611</v>
       </c>
-      <c r="V10" s="40" t="n">
+      <c r="V10" s="41" t="n">
         <v>0.0492611</v>
       </c>
     </row>
@@ -13717,14 +13717,14 @@
         <v>78.5</v>
       </c>
       <c r="N11" s="28" t="n">
-        <v>56.2</v>
-      </c>
-      <c r="O11" s="37" t="inlineStr">
+        <v>60.9</v>
+      </c>
+      <c r="O11" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P11" s="38" t="n">
+      <c r="P11" s="39" t="n">
         <v>34.2</v>
       </c>
       <c r="Q11" s="23" t="inlineStr">
@@ -13765,42 +13765,42 @@
       <c r="D12" s="26" t="n">
         <v>185.6</v>
       </c>
-      <c r="E12" s="39" t="n">
+      <c r="E12" s="40" t="n">
         <v>1.66</v>
       </c>
-      <c r="F12" s="40" t="n">
+      <c r="F12" s="41" t="n">
         <v>1.719</v>
       </c>
-      <c r="G12" s="40" t="n">
+      <c r="G12" s="41" t="n">
         <v>-1.797</v>
       </c>
-      <c r="H12" s="40" t="n">
+      <c r="H12" s="41" t="n">
         <v>0.508</v>
       </c>
-      <c r="I12" s="40" t="n">
+      <c r="I12" s="41" t="n">
         <v>-0.362</v>
       </c>
-      <c r="J12" s="40" t="n">
+      <c r="J12" s="41" t="n">
         <v>0.517</v>
       </c>
-      <c r="K12" s="41" t="n">
+      <c r="K12" s="42" t="n">
         <v>85</v>
       </c>
-      <c r="L12" s="41" t="n">
+      <c r="L12" s="42" t="n">
         <v>63.5</v>
       </c>
-      <c r="M12" s="42" t="n">
+      <c r="M12" s="43" t="n">
         <v>76.40000000000001</v>
       </c>
-      <c r="N12" s="28" t="n">
-        <v>61.7</v>
-      </c>
-      <c r="O12" s="43" t="inlineStr">
+      <c r="N12" s="37" t="n">
+        <v>50</v>
+      </c>
+      <c r="O12" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P12" s="38" t="n">
+      <c r="P12" s="39" t="n">
         <v>9.4</v>
       </c>
       <c r="Q12" s="23" t="inlineStr">
@@ -13808,19 +13808,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R12" s="40" t="n">
+      <c r="R12" s="41" t="n">
         <v>-0.2813853</v>
       </c>
-      <c r="S12" s="40" t="n">
+      <c r="S12" s="41" t="n">
         <v>0.4188034</v>
       </c>
-      <c r="T12" s="40" t="n">
+      <c r="T12" s="41" t="n">
         <v>-0.3112033</v>
       </c>
-      <c r="U12" s="40" t="n">
+      <c r="U12" s="41" t="n">
         <v>-0.1487179</v>
       </c>
-      <c r="V12" s="40" t="n">
+      <c r="V12" s="41" t="n">
         <v>-0.3615385</v>
       </c>
     </row>
@@ -13869,14 +13869,14 @@
         <v>75.59999999999999</v>
       </c>
       <c r="N13" s="28" t="n">
-        <v>53.6</v>
-      </c>
-      <c r="O13" s="37" t="inlineStr">
+        <v>59.3</v>
+      </c>
+      <c r="O13" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P13" s="38" t="n">
+      <c r="P13" s="39" t="n">
         <v>29.6</v>
       </c>
       <c r="Q13" s="23" t="inlineStr">
@@ -13917,62 +13917,62 @@
       <c r="D14" s="26" t="n">
         <v>134.3</v>
       </c>
-      <c r="E14" s="39" t="n">
+      <c r="E14" s="40" t="n">
         <v>5.92</v>
       </c>
-      <c r="F14" s="40" t="n">
+      <c r="F14" s="41" t="n">
         <v>0.109</v>
       </c>
-      <c r="G14" s="40" t="n">
+      <c r="G14" s="41" t="n">
         <v>-0.183</v>
       </c>
-      <c r="H14" s="40" t="n">
+      <c r="H14" s="41" t="n">
         <v>0.599</v>
       </c>
-      <c r="I14" s="40" t="n">
+      <c r="I14" s="41" t="n">
         <v>0.03700000000000001</v>
       </c>
-      <c r="J14" s="40" t="n">
+      <c r="J14" s="41" t="n">
         <v>0.217</v>
       </c>
-      <c r="K14" s="41" t="n">
+      <c r="K14" s="42" t="n">
         <v>62.2</v>
       </c>
-      <c r="L14" s="41" t="n">
+      <c r="L14" s="42" t="n">
         <v>91.5</v>
       </c>
-      <c r="M14" s="42" t="n">
+      <c r="M14" s="43" t="n">
         <v>73.90000000000001</v>
       </c>
-      <c r="N14" s="28" t="n">
-        <v>66.90000000000001</v>
-      </c>
-      <c r="O14" s="43" t="inlineStr">
+      <c r="N14" s="22" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="O14" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P14" s="38" t="n">
+      <c r="P14" s="39" t="n">
         <v>3.2</v>
       </c>
-      <c r="Q14" s="45" t="inlineStr">
+      <c r="Q14" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R14" s="40" t="n">
+      <c r="R14" s="41" t="n">
         <v>0.0942699</v>
       </c>
-      <c r="S14" s="40" t="n">
+      <c r="S14" s="41" t="n">
         <v>-0.5264</v>
       </c>
-      <c r="T14" s="40" t="n">
+      <c r="T14" s="41" t="n">
         <v>-0.6990341</v>
       </c>
-      <c r="U14" s="40" t="n">
+      <c r="U14" s="41" t="n">
         <v>-0.6474092</v>
       </c>
-      <c r="V14" s="40" t="n">
+      <c r="V14" s="41" t="n">
         <v>-0.7771922999999999</v>
       </c>
     </row>
@@ -14064,19 +14064,19 @@
           <t>KVHI</t>
         </is>
       </c>
-      <c r="B20" s="41" t="n">
+      <c r="B20" s="42" t="n">
         <v>54.4</v>
       </c>
-      <c r="C20" s="41" t="n">
+      <c r="C20" s="42" t="n">
         <v>72.2</v>
       </c>
-      <c r="D20" s="41" t="n">
+      <c r="D20" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E20" s="41" t="n">
+      <c r="E20" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="F20" s="41" t="n">
+      <c r="F20" s="42" t="n">
         <v>100</v>
       </c>
     </row>
@@ -14108,19 +14108,19 @@
           <t>CODA</t>
         </is>
       </c>
-      <c r="B22" s="41" t="n">
+      <c r="B22" s="42" t="n">
         <v>57.6</v>
       </c>
-      <c r="C22" s="41" t="n">
+      <c r="C22" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D22" s="41" t="n">
+      <c r="D22" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E22" s="41" t="n">
+      <c r="E22" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="F22" s="41" t="n">
+      <c r="F22" s="42" t="n">
         <v>100</v>
       </c>
     </row>
@@ -14152,19 +14152,19 @@
           <t>SCTQ</t>
         </is>
       </c>
-      <c r="B24" s="41" t="n">
+      <c r="B24" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="C24" s="41" t="n">
+      <c r="C24" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D24" s="41" t="n">
+      <c r="D24" s="42" t="n">
         <v>99.2</v>
       </c>
-      <c r="E24" s="41" t="n">
+      <c r="E24" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="F24" s="41" t="n">
+      <c r="F24" s="42" t="n">
         <v>50</v>
       </c>
     </row>
@@ -14196,19 +14196,19 @@
           <t>BZAI</t>
         </is>
       </c>
-      <c r="B26" s="41" t="n">
+      <c r="B26" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="C26" s="41" t="n">
+      <c r="C26" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D26" s="41" t="n">
+      <c r="D26" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E26" s="41" t="n">
+      <c r="E26" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="F26" s="41" t="n">
+      <c r="F26" s="42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14240,19 +14240,19 @@
           <t>BYRN</t>
         </is>
       </c>
-      <c r="B28" s="41" t="n">
+      <c r="B28" s="42" t="n">
         <v>21.8</v>
       </c>
-      <c r="C28" s="41" t="n">
+      <c r="C28" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D28" s="41" t="n">
+      <c r="D28" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E28" s="41" t="n">
+      <c r="E28" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="F28" s="41" t="n">
+      <c r="F28" s="42" t="n">
         <v>4.2</v>
       </c>
     </row>
@@ -14916,14 +14916,14 @@
         <v>82.59999999999999</v>
       </c>
       <c r="N5" s="28" t="n">
-        <v>65.59999999999999</v>
-      </c>
-      <c r="O5" s="37" t="inlineStr">
+        <v>58.8</v>
+      </c>
+      <c r="O5" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P5" s="38" t="n">
+      <c r="P5" s="39" t="n">
         <v>23.5</v>
       </c>
       <c r="Q5" s="23" t="inlineStr">
@@ -14964,42 +14964,42 @@
       <c r="D6" s="26" t="n">
         <v>1063</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="E6" s="40" t="n">
         <v>5.91</v>
       </c>
-      <c r="F6" s="40" t="n">
+      <c r="F6" s="41" t="n">
         <v>0.447</v>
       </c>
-      <c r="G6" s="40" t="n">
+      <c r="G6" s="41" t="n">
         <v>0.194</v>
       </c>
-      <c r="H6" s="40" t="n">
+      <c r="H6" s="41" t="n">
         <v>0.514</v>
       </c>
-      <c r="I6" s="40" t="n">
+      <c r="I6" s="41" t="n">
         <v>0.189</v>
       </c>
-      <c r="J6" s="40" t="n">
+      <c r="J6" s="41" t="n">
         <v>0.051</v>
       </c>
-      <c r="K6" s="41" t="n">
+      <c r="K6" s="42" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="L6" s="41" t="n">
+      <c r="L6" s="42" t="n">
         <v>87.8</v>
       </c>
-      <c r="M6" s="42" t="n">
+      <c r="M6" s="43" t="n">
         <v>82</v>
       </c>
-      <c r="N6" s="22" t="n">
-        <v>70.7</v>
-      </c>
-      <c r="O6" s="43" t="inlineStr">
+      <c r="N6" s="37" t="n">
+        <v>50</v>
+      </c>
+      <c r="O6" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P6" s="38" t="n">
+      <c r="P6" s="39" t="n">
         <v>12.4</v>
       </c>
       <c r="Q6" s="23" t="inlineStr">
@@ -15007,19 +15007,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R6" s="40" t="n">
+      <c r="R6" s="41" t="n">
         <v>-0.1825726</v>
       </c>
-      <c r="S6" s="40" t="n">
+      <c r="S6" s="41" t="n">
         <v>0.1387283</v>
       </c>
-      <c r="T6" s="40" t="n">
+      <c r="T6" s="41" t="n">
         <v>-0.113943</v>
       </c>
-      <c r="U6" s="40" t="n">
+      <c r="U6" s="41" t="n">
         <v>-0.174581</v>
       </c>
-      <c r="V6" s="40" t="n">
+      <c r="V6" s="41" t="n">
         <v>0.1150943</v>
       </c>
     </row>
@@ -15068,14 +15068,14 @@
         <v>81.7</v>
       </c>
       <c r="N7" s="28" t="n">
-        <v>66.09999999999999</v>
-      </c>
-      <c r="O7" s="37" t="inlineStr">
+        <v>67.8</v>
+      </c>
+      <c r="O7" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P7" s="44" t="n">
+      <c r="P7" s="45" t="n">
         <v>65.09999999999999</v>
       </c>
       <c r="Q7" s="23" t="inlineStr">
@@ -15116,42 +15116,42 @@
       <c r="D8" s="26" t="n">
         <v>370.2</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="E8" s="40" t="n">
         <v>12.88</v>
       </c>
-      <c r="F8" s="40" t="n">
+      <c r="F8" s="41" t="n">
         <v>3.578</v>
       </c>
-      <c r="G8" s="40" t="n">
+      <c r="G8" s="41" t="n">
         <v>3.548</v>
       </c>
-      <c r="H8" s="40" t="n">
+      <c r="H8" s="41" t="n">
         <v>0.281</v>
       </c>
-      <c r="I8" s="40" t="n">
+      <c r="I8" s="41" t="n">
         <v>0.002</v>
       </c>
-      <c r="J8" s="40" t="n">
+      <c r="J8" s="41" t="n">
         <v>0.028</v>
       </c>
-      <c r="K8" s="41" t="n">
+      <c r="K8" s="42" t="n">
         <v>83.2</v>
       </c>
-      <c r="L8" s="41" t="n">
+      <c r="L8" s="42" t="n">
         <v>78.2</v>
       </c>
-      <c r="M8" s="42" t="n">
+      <c r="M8" s="43" t="n">
         <v>81.2</v>
       </c>
-      <c r="N8" s="41" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="O8" s="43" t="inlineStr">
+      <c r="N8" s="42" t="n">
+        <v>47</v>
+      </c>
+      <c r="O8" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P8" s="38" t="n">
+      <c r="P8" s="39" t="n">
         <v>0.2</v>
       </c>
       <c r="Q8" s="23" t="inlineStr">
@@ -15159,19 +15159,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R8" s="40" t="n">
+      <c r="R8" s="41" t="n">
         <v>-0.1592689</v>
       </c>
-      <c r="S8" s="40" t="n">
+      <c r="S8" s="41" t="n">
         <v>-0.301897</v>
       </c>
-      <c r="T8" s="40" t="n">
+      <c r="T8" s="41" t="n">
         <v>-0.2489796</v>
       </c>
-      <c r="U8" s="40" t="n">
+      <c r="U8" s="41" t="n">
         <v>-0.2533333</v>
       </c>
-      <c r="V8" s="40" t="n">
+      <c r="V8" s="41" t="n">
         <v>-0.1326599</v>
       </c>
     </row>
@@ -15220,14 +15220,14 @@
         <v>79.5</v>
       </c>
       <c r="N9" s="35" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="O9" s="37" t="inlineStr">
+        <v>47.6</v>
+      </c>
+      <c r="O9" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P9" s="38" t="n">
+      <c r="P9" s="39" t="n">
         <v>8.199999999999999</v>
       </c>
       <c r="Q9" s="23" t="inlineStr">
@@ -15268,42 +15268,42 @@
       <c r="D10" s="26" t="n">
         <v>1243.3</v>
       </c>
-      <c r="E10" s="39" t="n">
+      <c r="E10" s="40" t="n">
         <v>15.35</v>
       </c>
-      <c r="F10" s="40" t="n">
+      <c r="F10" s="41" t="n">
         <v>0.155</v>
       </c>
-      <c r="G10" s="40" t="n">
+      <c r="G10" s="41" t="n">
         <v>0.059</v>
       </c>
-      <c r="H10" s="40" t="n">
+      <c r="H10" s="41" t="n">
         <v>0.395</v>
       </c>
-      <c r="I10" s="40" t="n">
+      <c r="I10" s="41" t="n">
         <v>0.025</v>
       </c>
-      <c r="J10" s="40" t="n">
+      <c r="J10" s="41" t="n">
         <v>0.08199999999999999</v>
       </c>
-      <c r="K10" s="41" t="n">
+      <c r="K10" s="42" t="n">
         <v>71.09999999999999</v>
       </c>
-      <c r="L10" s="41" t="n">
+      <c r="L10" s="42" t="n">
         <v>99.2</v>
       </c>
-      <c r="M10" s="42" t="n">
+      <c r="M10" s="43" t="n">
         <v>78.90000000000001</v>
       </c>
       <c r="N10" s="28" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="O10" s="43" t="inlineStr">
+        <v>54.4</v>
+      </c>
+      <c r="O10" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P10" s="44" t="n">
+      <c r="P10" s="45" t="n">
         <v>48.2</v>
       </c>
       <c r="Q10" s="23" t="inlineStr">
@@ -15311,19 +15311,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R10" s="40" t="n">
+      <c r="R10" s="41" t="n">
         <v>0.0032679739</v>
       </c>
-      <c r="S10" s="40" t="n">
+      <c r="S10" s="41" t="n">
         <v>0.5258449000000001</v>
       </c>
-      <c r="T10" s="40" t="n">
+      <c r="T10" s="41" t="n">
         <v>0.7995310999999999</v>
       </c>
-      <c r="U10" s="40" t="n">
+      <c r="U10" s="41" t="n">
         <v>0.7663982</v>
       </c>
-      <c r="V10" s="40" t="n">
+      <c r="V10" s="41" t="n">
         <v>0.9283920000000001</v>
       </c>
     </row>
@@ -15372,14 +15372,14 @@
         <v>76.7</v>
       </c>
       <c r="N11" s="28" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="O11" s="37" t="inlineStr">
+        <v>55.3</v>
+      </c>
+      <c r="O11" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P11" s="38" t="n">
+      <c r="P11" s="39" t="n">
         <v>34.5</v>
       </c>
       <c r="Q11" s="23" t="inlineStr">
@@ -15420,62 +15420,62 @@
       <c r="D12" s="26" t="n">
         <v>659.4</v>
       </c>
-      <c r="E12" s="39" t="n">
+      <c r="E12" s="40" t="n">
         <v>14.82</v>
       </c>
-      <c r="F12" s="40" t="n">
+      <c r="F12" s="41" t="n">
         <v>0.171</v>
       </c>
-      <c r="G12" s="40" t="n">
+      <c r="G12" s="41" t="n">
         <v>0.4429999999999999</v>
       </c>
-      <c r="H12" s="40" t="n">
+      <c r="H12" s="41" t="n">
         <v>0.262</v>
       </c>
-      <c r="I12" s="40" t="n">
+      <c r="I12" s="41" t="n">
         <v>-0.033</v>
       </c>
-      <c r="J12" s="40" t="n">
+      <c r="J12" s="41" t="n">
         <v>0.031</v>
       </c>
-      <c r="K12" s="41" t="n">
+      <c r="K12" s="42" t="n">
         <v>63</v>
       </c>
-      <c r="L12" s="41" t="n">
+      <c r="L12" s="42" t="n">
         <v>98.5</v>
       </c>
-      <c r="M12" s="42" t="n">
+      <c r="M12" s="43" t="n">
         <v>74.5</v>
       </c>
-      <c r="N12" s="41" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="O12" s="43" t="inlineStr">
+      <c r="N12" s="42" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="O12" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P12" s="44" t="n">
+      <c r="P12" s="45" t="n">
         <v>47.1</v>
       </c>
-      <c r="Q12" s="45" t="inlineStr">
+      <c r="Q12" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R12" s="40" t="n">
+      <c r="R12" s="41" t="n">
         <v>-0.0243581</v>
       </c>
-      <c r="S12" s="40" t="n">
+      <c r="S12" s="41" t="n">
         <v>0.2569975</v>
       </c>
-      <c r="T12" s="40" t="n">
+      <c r="T12" s="41" t="n">
         <v>0.3521898</v>
       </c>
-      <c r="U12" s="40" t="n">
+      <c r="U12" s="41" t="n">
         <v>0.5015198000000001</v>
       </c>
-      <c r="V12" s="40" t="n">
+      <c r="V12" s="41" t="n">
         <v>0.5278351</v>
       </c>
     </row>
@@ -15524,17 +15524,17 @@
         <v>74.3</v>
       </c>
       <c r="N13" s="35" t="n">
-        <v>44.7</v>
-      </c>
-      <c r="O13" s="37" t="inlineStr">
+        <v>47.5</v>
+      </c>
+      <c r="O13" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P13" s="38" t="n">
+      <c r="P13" s="39" t="n">
         <v>4.1</v>
       </c>
-      <c r="Q13" s="45" t="inlineStr">
+      <c r="Q13" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -15572,62 +15572,62 @@
       <c r="D14" s="26" t="n">
         <v>321.6</v>
       </c>
-      <c r="E14" s="39" t="n">
+      <c r="E14" s="40" t="n">
         <v>4.02</v>
       </c>
-      <c r="F14" s="40" t="n">
+      <c r="F14" s="41" t="n">
         <v>0.271</v>
       </c>
-      <c r="G14" s="40" t="n">
+      <c r="G14" s="41" t="n">
         <v>0.335</v>
       </c>
-      <c r="H14" s="40" t="n">
+      <c r="H14" s="41" t="n">
         <v>0.5379999999999999</v>
       </c>
-      <c r="I14" s="40" t="n">
+      <c r="I14" s="41" t="n">
         <v>-0.165</v>
       </c>
-      <c r="J14" s="40" t="n">
+      <c r="J14" s="41" t="n">
         <v>0.328</v>
       </c>
-      <c r="K14" s="41" t="n">
+      <c r="K14" s="42" t="n">
         <v>86.3</v>
       </c>
-      <c r="L14" s="41" t="n">
+      <c r="L14" s="42" t="n">
         <v>94.7</v>
       </c>
-      <c r="M14" s="42" t="n">
+      <c r="M14" s="43" t="n">
         <v>74.2</v>
       </c>
       <c r="N14" s="28" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="O14" s="43" t="inlineStr">
+        <v>62.1</v>
+      </c>
+      <c r="O14" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P14" s="46" t="n">
+      <c r="P14" s="37" t="n">
         <v>72.3</v>
       </c>
-      <c r="Q14" s="45" t="inlineStr">
+      <c r="Q14" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R14" s="40" t="n">
+      <c r="R14" s="41" t="n">
         <v>-0.012285</v>
       </c>
-      <c r="S14" s="40" t="n">
+      <c r="S14" s="41" t="n">
         <v>0.1858407</v>
       </c>
-      <c r="T14" s="40" t="n">
+      <c r="T14" s="41" t="n">
         <v>0.6890756</v>
       </c>
-      <c r="U14" s="40" t="n">
+      <c r="U14" s="41" t="n">
         <v>0.3267327</v>
       </c>
-      <c r="V14" s="40" t="n">
+      <c r="V14" s="41" t="n">
         <v>1.4662577</v>
       </c>
     </row>
@@ -15719,19 +15719,19 @@
           <t>EVLV</t>
         </is>
       </c>
-      <c r="B20" s="41" t="n">
+      <c r="B20" s="42" t="n">
         <v>89.40000000000001</v>
       </c>
-      <c r="C20" s="41" t="n">
+      <c r="C20" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D20" s="41" t="n">
+      <c r="D20" s="42" t="n">
         <v>44.4</v>
       </c>
-      <c r="E20" s="41" t="n">
+      <c r="E20" s="42" t="n">
         <v>51</v>
       </c>
-      <c r="F20" s="41" t="n">
+      <c r="F20" s="42" t="n">
         <v>98.5</v>
       </c>
     </row>
@@ -15763,19 +15763,19 @@
           <t>CMCO</t>
         </is>
       </c>
-      <c r="B22" s="41" t="n">
+      <c r="B22" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="C22" s="41" t="n">
+      <c r="C22" s="42" t="n">
         <v>70.2</v>
       </c>
-      <c r="D22" s="41" t="n">
+      <c r="D22" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E22" s="41" t="n">
+      <c r="E22" s="42" t="n">
         <v>28</v>
       </c>
-      <c r="F22" s="41" t="n">
+      <c r="F22" s="42" t="n">
         <v>100</v>
       </c>
     </row>
@@ -15807,19 +15807,19 @@
           <t>ADTN</t>
         </is>
       </c>
-      <c r="B24" s="41" t="n">
+      <c r="B24" s="42" t="n">
         <v>31</v>
       </c>
-      <c r="C24" s="41" t="n">
+      <c r="C24" s="42" t="n">
         <v>98.8</v>
       </c>
-      <c r="D24" s="41" t="n">
+      <c r="D24" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E24" s="41" t="n">
+      <c r="E24" s="42" t="n">
         <v>82</v>
       </c>
-      <c r="F24" s="41" t="n">
+      <c r="F24" s="42" t="n">
         <v>64.8</v>
       </c>
     </row>
@@ -15851,19 +15851,19 @@
           <t>SWBI</t>
         </is>
       </c>
-      <c r="B26" s="41" t="n">
+      <c r="B26" s="42" t="n">
         <v>34.2</v>
       </c>
-      <c r="C26" s="41" t="n">
+      <c r="C26" s="42" t="n">
         <v>65.5</v>
       </c>
-      <c r="D26" s="41" t="n">
+      <c r="D26" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E26" s="41" t="n">
+      <c r="E26" s="42" t="n">
         <v>31</v>
       </c>
-      <c r="F26" s="41" t="n">
+      <c r="F26" s="42" t="n">
         <v>100</v>
       </c>
     </row>
@@ -15895,19 +15895,19 @@
           <t>BUKS</t>
         </is>
       </c>
-      <c r="B28" s="41" t="n">
+      <c r="B28" s="42" t="n">
         <v>54.2</v>
       </c>
-      <c r="C28" s="41" t="n">
+      <c r="C28" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D28" s="41" t="n">
+      <c r="D28" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E28" s="41" t="n">
+      <c r="E28" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="F28" s="41" t="n">
+      <c r="F28" s="42" t="n">
         <v>100</v>
       </c>
     </row>
@@ -16573,12 +16573,12 @@
       <c r="N5" s="28" t="n">
         <v>65.8</v>
       </c>
-      <c r="O5" s="37" t="inlineStr">
+      <c r="O5" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P5" s="38" t="n">
+      <c r="P5" s="39" t="n">
         <v>6.8</v>
       </c>
       <c r="Q5" s="23" t="inlineStr">
@@ -16619,42 +16619,42 @@
       <c r="D6" s="26" t="n">
         <v>9705.299999999999</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="E6" s="40" t="n">
         <v>39.84</v>
       </c>
-      <c r="F6" s="40" t="n">
+      <c r="F6" s="41" t="n">
         <v>0.415</v>
       </c>
-      <c r="G6" s="40" t="n">
+      <c r="G6" s="41" t="n">
         <v>0.446</v>
       </c>
-      <c r="H6" s="40" t="n">
+      <c r="H6" s="41" t="n">
         <v>0.384</v>
       </c>
-      <c r="I6" s="40" t="n">
+      <c r="I6" s="41" t="n">
         <v>0.006999999999999999</v>
       </c>
-      <c r="J6" s="40" t="n">
+      <c r="J6" s="41" t="n">
         <v>0.064</v>
       </c>
-      <c r="K6" s="41" t="n">
+      <c r="K6" s="42" t="n">
         <v>88.7</v>
       </c>
-      <c r="L6" s="41" t="n">
+      <c r="L6" s="42" t="n">
         <v>80</v>
       </c>
-      <c r="M6" s="42" t="n">
+      <c r="M6" s="43" t="n">
         <v>79.8</v>
       </c>
-      <c r="N6" s="41" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="O6" s="43" t="inlineStr">
+      <c r="N6" s="28" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="O6" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P6" s="44" t="n">
+      <c r="P6" s="45" t="n">
         <v>52.7</v>
       </c>
       <c r="Q6" s="23" t="inlineStr">
@@ -16662,19 +16662,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R6" s="40" t="n">
+      <c r="R6" s="41" t="n">
         <v>-0.09433960000000001</v>
       </c>
-      <c r="S6" s="40" t="n">
+      <c r="S6" s="41" t="n">
         <v>0.2032619</v>
       </c>
-      <c r="T6" s="40" t="n">
+      <c r="T6" s="41" t="n">
         <v>0.5096628</v>
       </c>
-      <c r="U6" s="40" t="n">
+      <c r="U6" s="41" t="n">
         <v>0.5942377</v>
       </c>
-      <c r="V6" s="40" t="n">
+      <c r="V6" s="41" t="n">
         <v>0.8739417</v>
       </c>
     </row>
@@ -16723,14 +16723,14 @@
         <v>77.59999999999999</v>
       </c>
       <c r="N7" s="28" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="O7" s="37" t="inlineStr">
+        <v>53.3</v>
+      </c>
+      <c r="O7" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P7" s="38" t="n">
+      <c r="P7" s="39" t="n">
         <v>39.7</v>
       </c>
       <c r="Q7" s="23" t="inlineStr">
@@ -16771,42 +16771,42 @@
       <c r="D8" s="26" t="n">
         <v>5182.7</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="E8" s="40" t="n">
         <v>13.65</v>
       </c>
-      <c r="F8" s="40" t="n">
+      <c r="F8" s="41" t="n">
         <v>0.138</v>
       </c>
-      <c r="G8" s="40" t="n">
+      <c r="G8" s="41" t="n">
         <v>0.128</v>
       </c>
-      <c r="H8" s="40" t="n">
+      <c r="H8" s="41" t="n">
         <v>0.476</v>
       </c>
-      <c r="I8" s="40" t="n">
+      <c r="I8" s="41" t="n">
         <v>0.035</v>
       </c>
-      <c r="J8" s="40" t="n">
+      <c r="J8" s="41" t="n">
         <v>0.13</v>
       </c>
-      <c r="K8" s="41" t="n">
+      <c r="K8" s="42" t="n">
         <v>75.59999999999999</v>
       </c>
-      <c r="L8" s="41" t="n">
+      <c r="L8" s="42" t="n">
         <v>80</v>
       </c>
-      <c r="M8" s="42" t="n">
+      <c r="M8" s="43" t="n">
         <v>77.40000000000001</v>
       </c>
-      <c r="N8" s="41" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="O8" s="43" t="inlineStr">
+      <c r="N8" s="42" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="O8" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P8" s="38" t="n">
+      <c r="P8" s="39" t="n">
         <v>4</v>
       </c>
       <c r="Q8" s="23" t="inlineStr">
@@ -16814,19 +16814,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R8" s="40" t="n">
+      <c r="R8" s="41" t="n">
         <v>-0.0312278</v>
       </c>
-      <c r="S8" s="40" t="n">
+      <c r="S8" s="41" t="n">
         <v>0.0356601</v>
       </c>
-      <c r="T8" s="40" t="n">
+      <c r="T8" s="41" t="n">
         <v>-0.4057466</v>
       </c>
-      <c r="U8" s="40" t="n">
+      <c r="U8" s="41" t="n">
         <v>-0.295302</v>
       </c>
-      <c r="V8" s="40" t="n">
+      <c r="V8" s="41" t="n">
         <v>-0.121056</v>
       </c>
     </row>
@@ -16875,14 +16875,14 @@
         <v>75.8</v>
       </c>
       <c r="N9" s="28" t="n">
-        <v>51.5</v>
-      </c>
-      <c r="O9" s="37" t="inlineStr">
+        <v>54.2</v>
+      </c>
+      <c r="O9" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P9" s="38" t="n">
+      <c r="P9" s="39" t="n">
         <v>27</v>
       </c>
       <c r="Q9" s="23" t="inlineStr">
@@ -16923,42 +16923,42 @@
       <c r="D10" s="26" t="n">
         <v>8638.799999999999</v>
       </c>
-      <c r="E10" s="39" t="n">
+      <c r="E10" s="40" t="n">
         <v>46.39</v>
       </c>
-      <c r="F10" s="40" t="n">
+      <c r="F10" s="41" t="n">
         <v>0.261</v>
       </c>
-      <c r="G10" s="40" t="n">
+      <c r="G10" s="41" t="n">
         <v>0.106</v>
       </c>
-      <c r="H10" s="40" t="n">
+      <c r="H10" s="41" t="n">
         <v>0.471</v>
       </c>
-      <c r="I10" s="40" t="n">
+      <c r="I10" s="41" t="n">
         <v>-0.035</v>
       </c>
-      <c r="J10" s="40" t="n">
+      <c r="J10" s="41" t="n">
         <v>0.334</v>
       </c>
-      <c r="K10" s="41" t="n">
+      <c r="K10" s="42" t="n">
         <v>82.09999999999999</v>
       </c>
-      <c r="L10" s="41" t="n">
+      <c r="L10" s="42" t="n">
         <v>77.3</v>
       </c>
-      <c r="M10" s="42" t="n">
+      <c r="M10" s="43" t="n">
         <v>75</v>
       </c>
       <c r="N10" s="28" t="n">
-        <v>50.3</v>
-      </c>
-      <c r="O10" s="43" t="inlineStr">
+        <v>53.1</v>
+      </c>
+      <c r="O10" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P10" s="44" t="n">
+      <c r="P10" s="45" t="n">
         <v>52.9</v>
       </c>
       <c r="Q10" s="23" t="inlineStr">
@@ -16966,19 +16966,19 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="R10" s="40" t="n">
+      <c r="R10" s="41" t="n">
         <v>-0.0662238</v>
       </c>
-      <c r="S10" s="40" t="n">
+      <c r="S10" s="41" t="n">
         <v>0.4151922</v>
       </c>
-      <c r="T10" s="40" t="n">
+      <c r="T10" s="41" t="n">
         <v>0.5876112</v>
       </c>
-      <c r="U10" s="40" t="n">
+      <c r="U10" s="41" t="n">
         <v>0.7585292</v>
       </c>
-      <c r="V10" s="40" t="n">
+      <c r="V10" s="41" t="n">
         <v>0.6597495999999999</v>
       </c>
     </row>
@@ -17026,18 +17026,18 @@
       <c r="M11" s="36" t="n">
         <v>72.90000000000001</v>
       </c>
-      <c r="N11" s="28" t="n">
-        <v>68</v>
-      </c>
-      <c r="O11" s="37" t="inlineStr">
+      <c r="N11" s="22" t="n">
+        <v>76</v>
+      </c>
+      <c r="O11" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P11" s="44" t="n">
+      <c r="P11" s="45" t="n">
         <v>51.9</v>
       </c>
-      <c r="Q11" s="45" t="inlineStr">
+      <c r="Q11" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -17075,62 +17075,62 @@
       <c r="D12" s="26" t="n">
         <v>5354.5</v>
       </c>
-      <c r="E12" s="39" t="n">
+      <c r="E12" s="40" t="n">
         <v>87.95</v>
       </c>
-      <c r="F12" s="40" t="n">
+      <c r="F12" s="41" t="n">
         <v>0.099</v>
       </c>
-      <c r="G12" s="40" t="n">
+      <c r="G12" s="41" t="n">
         <v>0.14</v>
       </c>
-      <c r="H12" s="40" t="n">
+      <c r="H12" s="41" t="n">
         <v>0.369</v>
       </c>
-      <c r="I12" s="40" t="n">
+      <c r="I12" s="41" t="n">
         <v>0.012</v>
       </c>
-      <c r="J12" s="40" t="n">
+      <c r="J12" s="41" t="n">
         <v>0.066</v>
       </c>
-      <c r="K12" s="41" t="n">
+      <c r="K12" s="42" t="n">
         <v>67</v>
       </c>
-      <c r="L12" s="41" t="n">
+      <c r="L12" s="42" t="n">
         <v>79.5</v>
       </c>
-      <c r="M12" s="42" t="n">
+      <c r="M12" s="43" t="n">
         <v>72</v>
       </c>
-      <c r="N12" s="41" t="n">
-        <v>46.6</v>
-      </c>
-      <c r="O12" s="43" t="inlineStr">
+      <c r="N12" s="42" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="O12" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P12" s="38" t="n">
+      <c r="P12" s="39" t="n">
         <v>5.3</v>
       </c>
-      <c r="Q12" s="45" t="inlineStr">
+      <c r="Q12" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R12" s="40" t="n">
+      <c r="R12" s="41" t="n">
         <v>-0.09544380000000001</v>
       </c>
-      <c r="S12" s="40" t="n">
+      <c r="S12" s="41" t="n">
         <v>-0.2244268</v>
       </c>
-      <c r="T12" s="40" t="n">
+      <c r="T12" s="41" t="n">
         <v>-0.2051514</v>
       </c>
-      <c r="U12" s="40" t="n">
+      <c r="U12" s="41" t="n">
         <v>-0.2127641</v>
       </c>
-      <c r="V12" s="40" t="n">
+      <c r="V12" s="41" t="n">
         <v>-0.3001512</v>
       </c>
     </row>
@@ -17179,17 +17179,17 @@
         <v>71.90000000000001</v>
       </c>
       <c r="N13" s="35" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="O13" s="37" t="inlineStr">
+        <v>39.5</v>
+      </c>
+      <c r="O13" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P13" s="38" t="n">
+      <c r="P13" s="39" t="n">
         <v>15.5</v>
       </c>
-      <c r="Q13" s="45" t="inlineStr">
+      <c r="Q13" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -17227,62 +17227,62 @@
       <c r="D14" s="26" t="n">
         <v>10974.2</v>
       </c>
-      <c r="E14" s="39" t="n">
+      <c r="E14" s="40" t="n">
         <v>98.37</v>
       </c>
-      <c r="F14" s="40" t="n">
+      <c r="F14" s="41" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="G14" s="40" t="n">
+      <c r="G14" s="41" t="n">
         <v>0.109</v>
       </c>
-      <c r="H14" s="40" t="n">
+      <c r="H14" s="41" t="n">
         <v>0.545</v>
       </c>
-      <c r="I14" s="40" t="n">
+      <c r="I14" s="41" t="n">
         <v>-0.107</v>
       </c>
-      <c r="J14" s="40" t="n">
+      <c r="J14" s="41" t="n">
         <v>0.08400000000000001</v>
       </c>
-      <c r="K14" s="41" t="n">
+      <c r="K14" s="42" t="n">
         <v>68.40000000000001</v>
       </c>
-      <c r="L14" s="41" t="n">
+      <c r="L14" s="42" t="n">
         <v>75.2</v>
       </c>
-      <c r="M14" s="42" t="n">
+      <c r="M14" s="43" t="n">
         <v>71.09999999999999</v>
       </c>
-      <c r="N14" s="41" t="n">
-        <v>36.3</v>
-      </c>
-      <c r="O14" s="43" t="inlineStr">
+      <c r="N14" s="42" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="O14" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P14" s="38" t="n">
+      <c r="P14" s="39" t="n">
         <v>25.7</v>
       </c>
-      <c r="Q14" s="45" t="inlineStr">
+      <c r="Q14" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R14" s="40" t="n">
+      <c r="R14" s="41" t="n">
         <v>0.0657638</v>
       </c>
-      <c r="S14" s="40" t="n">
+      <c r="S14" s="41" t="n">
         <v>0.0186393</v>
       </c>
-      <c r="T14" s="40" t="n">
+      <c r="T14" s="41" t="n">
         <v>-0.0240103</v>
       </c>
-      <c r="U14" s="40" t="n">
+      <c r="U14" s="41" t="n">
         <v>0.0167442</v>
       </c>
-      <c r="V14" s="40" t="n">
+      <c r="V14" s="41" t="n">
         <v>0.08696130000000001</v>
       </c>
     </row>
@@ -17374,19 +17374,19 @@
           <t>ESI</t>
         </is>
       </c>
-      <c r="B20" s="41" t="n">
+      <c r="B20" s="42" t="n">
         <v>83</v>
       </c>
-      <c r="C20" s="41" t="n">
+      <c r="C20" s="42" t="n">
         <v>96</v>
       </c>
-      <c r="D20" s="41" t="n">
+      <c r="D20" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E20" s="41" t="n">
+      <c r="E20" s="42" t="n">
         <v>64</v>
       </c>
-      <c r="F20" s="41" t="n">
+      <c r="F20" s="42" t="n">
         <v>100</v>
       </c>
     </row>
@@ -17418,19 +17418,19 @@
           <t>LYFT</t>
         </is>
       </c>
-      <c r="B22" s="41" t="n">
+      <c r="B22" s="42" t="n">
         <v>27.6</v>
       </c>
-      <c r="C22" s="41" t="n">
+      <c r="C22" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D22" s="41" t="n">
+      <c r="D22" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E22" s="41" t="n">
+      <c r="E22" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="F22" s="41" t="n">
+      <c r="F22" s="42" t="n">
         <v>82</v>
       </c>
     </row>
@@ -17462,19 +17462,19 @@
           <t>ALGM</t>
         </is>
       </c>
-      <c r="B24" s="41" t="n">
+      <c r="B24" s="42" t="n">
         <v>52.2</v>
       </c>
-      <c r="C24" s="41" t="n">
+      <c r="C24" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D24" s="41" t="n">
+      <c r="D24" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E24" s="41" t="n">
+      <c r="E24" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="F24" s="41" t="n">
+      <c r="F24" s="42" t="n">
         <v>76.5</v>
       </c>
     </row>
@@ -17506,19 +17506,19 @@
           <t>ESAB</t>
         </is>
       </c>
-      <c r="B26" s="41" t="n">
+      <c r="B26" s="42" t="n">
         <v>19.8</v>
       </c>
-      <c r="C26" s="41" t="n">
+      <c r="C26" s="42" t="n">
         <v>92.2</v>
       </c>
-      <c r="D26" s="41" t="n">
+      <c r="D26" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E26" s="41" t="n">
+      <c r="E26" s="42" t="n">
         <v>66</v>
       </c>
-      <c r="F26" s="41" t="n">
+      <c r="F26" s="42" t="n">
         <v>85</v>
       </c>
     </row>
@@ -17550,19 +17550,19 @@
           <t>RVTY</t>
         </is>
       </c>
-      <c r="B28" s="41" t="n">
+      <c r="B28" s="42" t="n">
         <v>14</v>
       </c>
-      <c r="C28" s="41" t="n">
+      <c r="C28" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="D28" s="41" t="n">
+      <c r="D28" s="42" t="n">
         <v>100</v>
       </c>
-      <c r="E28" s="41" t="n">
+      <c r="E28" s="42" t="n">
         <v>84</v>
       </c>
-      <c r="F28" s="41" t="n">
+      <c r="F28" s="42" t="n">
         <v>77.2</v>
       </c>
     </row>
@@ -20449,7 +20449,7 @@
           <t>KVH Industries, Inc.</t>
         </is>
       </c>
-      <c r="E7" s="41" t="n">
+      <c r="E7" s="42" t="n">
         <v>86.8</v>
       </c>
       <c r="F7" s="50" t="inlineStr">
@@ -20475,7 +20475,7 @@
           <t>Blaize Holdings, Inc.</t>
         </is>
       </c>
-      <c r="L7" s="41" t="n">
+      <c r="L7" s="42" t="n">
         <v>-36.2</v>
       </c>
       <c r="M7" s="50" t="inlineStr">
@@ -20557,7 +20557,7 @@
           <t>Viant Technology Inc.</t>
         </is>
       </c>
-      <c r="E9" s="41" t="n">
+      <c r="E9" s="42" t="n">
         <v>82.59999999999999</v>
       </c>
       <c r="F9" s="50" t="inlineStr">
@@ -20583,7 +20583,7 @@
           <t>Westell Technologies, Inc.</t>
         </is>
       </c>
-      <c r="L9" s="41" t="n">
+      <c r="L9" s="42" t="n">
         <v>-11.3</v>
       </c>
       <c r="M9" s="50" t="inlineStr">
@@ -20803,7 +20803,7 @@
           <t>ADTRAN Holdings, Inc.</t>
         </is>
       </c>
-      <c r="E15" s="41" t="n">
+      <c r="E15" s="42" t="n">
         <v>99.2</v>
       </c>
       <c r="F15" s="50" t="inlineStr">
@@ -20829,7 +20829,7 @@
           <t>WhiteFiber, Inc. Ordinary Shares</t>
         </is>
       </c>
-      <c r="L15" s="41" t="n">
+      <c r="L15" s="42" t="n">
         <v>75.3</v>
       </c>
       <c r="M15" s="50" t="inlineStr">
@@ -20911,7 +20911,7 @@
           <t>Westell Technologies, Inc.</t>
         </is>
       </c>
-      <c r="E17" s="41" t="n">
+      <c r="E17" s="42" t="n">
         <v>98.59999999999999</v>
       </c>
       <c r="F17" s="50" t="inlineStr">
@@ -20937,7 +20937,7 @@
           <t>Coda Octopus Group, Inc.</t>
         </is>
       </c>
-      <c r="L17" s="41" t="n">
+      <c r="L17" s="42" t="n">
         <v>49.1</v>
       </c>
       <c r="M17" s="50" t="inlineStr">
@@ -21157,7 +21157,7 @@
           <t>Columbus McKinnon Corporation</t>
         </is>
       </c>
-      <c r="E23" s="41" t="n">
+      <c r="E23" s="42" t="n">
         <v>357.8</v>
       </c>
       <c r="F23" s="50" t="inlineStr">
@@ -21265,7 +21265,7 @@
           <t>KULR Technology Group, Inc.</t>
         </is>
       </c>
-      <c r="E25" s="41" t="n">
+      <c r="E25" s="42" t="n">
         <v>97.90000000000001</v>
       </c>
       <c r="F25" s="50" t="inlineStr">
@@ -21445,7 +21445,7 @@
           <t>Westell Technologies, Inc.</t>
         </is>
       </c>
-      <c r="E31" s="41" t="n">
+      <c r="E31" s="42" t="n">
         <v>49.8994</v>
       </c>
       <c r="F31" s="50" t="inlineStr">
@@ -21501,7 +21501,7 @@
           <t>Blaize Holdings, Inc.</t>
         </is>
       </c>
-      <c r="E33" s="41" t="n">
+      <c r="E33" s="42" t="n">
         <v>41.88034</v>
       </c>
       <c r="F33" s="50" t="inlineStr">
@@ -21753,7 +21753,7 @@
           <t>Fingerprint Match</t>
         </is>
       </c>
-      <c r="F7" s="41" t="n">
+      <c r="F7" s="42" t="n">
         <v>86.8</v>
       </c>
       <c r="G7" s="51" t="inlineStr">
@@ -21849,7 +21849,7 @@
           <t>Fingerprint Match</t>
         </is>
       </c>
-      <c r="F9" s="41" t="n">
+      <c r="F9" s="42" t="n">
         <v>82.59999999999999</v>
       </c>
       <c r="G9" s="51" t="inlineStr">
@@ -21945,7 +21945,7 @@
           <t>Fingerprint Match</t>
         </is>
       </c>
-      <c r="F11" s="41" t="n">
+      <c r="F11" s="42" t="n">
         <v>81.7</v>
       </c>
       <c r="G11" s="51" t="inlineStr">
@@ -22039,7 +22039,7 @@
           <t>Growth Inflection</t>
         </is>
       </c>
-      <c r="F13" s="41" t="n">
+      <c r="F13" s="42" t="n">
         <v>81.2</v>
       </c>
       <c r="G13" s="51" t="inlineStr">
@@ -22135,7 +22135,7 @@
           <t>High-Growth Quality</t>
         </is>
       </c>
-      <c r="F15" s="41" t="n">
+      <c r="F15" s="42" t="n">
         <v>80.7</v>
       </c>
       <c r="G15" s="51" t="inlineStr">
@@ -22232,7 +22232,7 @@
           <t>Fingerprint Match</t>
         </is>
       </c>
-      <c r="F17" s="41" t="n">
+      <c r="F17" s="42" t="n">
         <v>79.8</v>
       </c>
       <c r="G17" s="51" t="inlineStr">
@@ -22327,7 +22327,7 @@
           <t>Momentum Breakout</t>
         </is>
       </c>
-      <c r="F19" s="41" t="n">
+      <c r="F19" s="42" t="n">
         <v>78.90000000000001</v>
       </c>
       <c r="G19" s="51" t="inlineStr">
@@ -22422,7 +22422,7 @@
           <t>Growth Inflection</t>
         </is>
       </c>
-      <c r="F21" s="41" t="n">
+      <c r="F21" s="42" t="n">
         <v>77.59999999999999</v>
       </c>
       <c r="G21" s="51" t="inlineStr">
@@ -22514,7 +22514,7 @@
           <t>Insider Conviction</t>
         </is>
       </c>
-      <c r="F23" s="41" t="n">
+      <c r="F23" s="42" t="n">
         <v>76.7</v>
       </c>
       <c r="G23" s="51" t="inlineStr">
@@ -22612,7 +22612,7 @@
           <t>Emerging Watch</t>
         </is>
       </c>
-      <c r="F25" s="41" t="n">
+      <c r="F25" s="42" t="n">
         <v>75.8</v>
       </c>
       <c r="G25" s="51" t="inlineStr">
@@ -22707,7 +22707,7 @@
           <t>Insider Conviction</t>
         </is>
       </c>
-      <c r="F27" s="41" t="n">
+      <c r="F27" s="42" t="n">
         <v>75</v>
       </c>
       <c r="G27" s="51" t="inlineStr">
@@ -22746,7 +22746,7 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="D28" s="45" t="inlineStr">
+      <c r="D28" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -22793,7 +22793,7 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="D29" s="45" t="inlineStr">
+      <c r="D29" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -22803,7 +22803,7 @@
           <t>Fingerprint Match</t>
         </is>
       </c>
-      <c r="F29" s="41" t="n">
+      <c r="F29" s="42" t="n">
         <v>74.3</v>
       </c>
       <c r="G29" s="51" t="inlineStr">
@@ -22841,7 +22841,7 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="D30" s="45" t="inlineStr">
+      <c r="D30" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -22890,7 +22890,7 @@
           <t>Nano Cap</t>
         </is>
       </c>
-      <c r="D31" s="45" t="inlineStr">
+      <c r="D31" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -22900,7 +22900,7 @@
           <t>Insider Conviction</t>
         </is>
       </c>
-      <c r="F31" s="41" t="n">
+      <c r="F31" s="42" t="n">
         <v>73.90000000000001</v>
       </c>
       <c r="G31" s="51" t="inlineStr">
@@ -22939,7 +22939,7 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="D32" s="45" t="inlineStr">
+      <c r="D32" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -22986,7 +22986,7 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="D33" s="45" t="inlineStr">
+      <c r="D33" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -22996,7 +22996,7 @@
           <t>Emerging Watch</t>
         </is>
       </c>
-      <c r="F33" s="41" t="n">
+      <c r="F33" s="42" t="n">
         <v>72</v>
       </c>
       <c r="G33" s="51" t="inlineStr">
@@ -23032,7 +23032,7 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="D34" s="45" t="inlineStr">
+      <c r="D34" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -23079,7 +23079,7 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="D35" s="45" t="inlineStr">
+      <c r="D35" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -23089,7 +23089,7 @@
           <t>Emerging Watch</t>
         </is>
       </c>
-      <c r="F35" s="41" t="n">
+      <c r="F35" s="42" t="n">
         <v>71.09999999999999</v>
       </c>
       <c r="G35" s="51" t="inlineStr">
@@ -23510,7 +23510,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="F14" s="40" t="n">
+      <c r="F14" s="41" t="n">
         <v>0.08</v>
       </c>
       <c r="G14" s="76" t="n">
@@ -23588,7 +23588,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F16" s="40" t="n">
+      <c r="F16" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G16" s="76" t="n">
@@ -23662,7 +23662,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F18" s="40" t="n">
+      <c r="F18" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G18" s="76" t="n">
@@ -23740,7 +23740,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F20" s="40" t="n">
+      <c r="F20" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G20" s="76" t="n">
@@ -23818,7 +23818,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F22" s="40" t="n">
+      <c r="F22" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G22" s="76" t="n">
@@ -23896,7 +23896,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F24" s="40" t="n">
+      <c r="F24" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G24" s="76" t="n">
@@ -23974,7 +23974,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F26" s="40" t="n">
+      <c r="F26" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G26" s="76" t="n">
@@ -24048,7 +24048,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F28" s="40" t="n">
+      <c r="F28" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G28" s="76" t="n">
@@ -24126,7 +24126,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F30" s="40" t="n">
+      <c r="F30" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G30" s="76" t="n">
@@ -24200,7 +24200,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F32" s="40" t="n">
+      <c r="F32" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G32" s="76" t="n">
@@ -24278,7 +24278,7 @@
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="F34" s="40" t="n">
+      <c r="F34" s="41" t="n">
         <v>0.05</v>
       </c>
       <c r="G34" s="76" t="n">
@@ -24312,7 +24312,7 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E35" s="45" t="inlineStr">
+      <c r="E35" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -24351,12 +24351,12 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E36" s="45" t="inlineStr">
+      <c r="E36" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F36" s="40" t="n">
+      <c r="F36" s="41" t="n">
         <v>0.03</v>
       </c>
       <c r="G36" s="76" t="n">
@@ -24390,7 +24390,7 @@
           <t>Small Cap</t>
         </is>
       </c>
-      <c r="E37" s="45" t="inlineStr">
+      <c r="E37" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -24429,12 +24429,12 @@
           <t>Nano Cap</t>
         </is>
       </c>
-      <c r="E38" s="45" t="inlineStr">
+      <c r="E38" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F38" s="40" t="n">
+      <c r="F38" s="41" t="n">
         <v>0.03</v>
       </c>
       <c r="G38" s="76" t="n">
@@ -24468,7 +24468,7 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E39" s="45" t="inlineStr">
+      <c r="E39" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -24507,12 +24507,12 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E40" s="45" t="inlineStr">
+      <c r="E40" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F40" s="40" t="n">
+      <c r="F40" s="41" t="n">
         <v>0.03</v>
       </c>
       <c r="G40" s="76" t="n">
@@ -24546,7 +24546,7 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E41" s="45" t="inlineStr">
+      <c r="E41" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -24585,12 +24585,12 @@
           <t>Breakout</t>
         </is>
       </c>
-      <c r="E42" s="45" t="inlineStr">
+      <c r="E42" s="46" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F42" s="40" t="n">
+      <c r="F42" s="41" t="n">
         <v>0.03</v>
       </c>
       <c r="G42" s="76" t="n">

</xml_diff>